<commit_message>
planilha com dados atualizada corretamente
</commit_message>
<xml_diff>
--- a/Database/SPMEDICALGROUP.xlsx
+++ b/Database/SPMEDICALGROUP.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robertsena-mtz\Videos\ROBERT\SPMedicalGroup_2.0\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bart\Desktop\SPMedicalGroup_2.0\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA3E1CB-E3C0-494B-8970-2BCA83168206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53BFAD26-ECE9-475F-89DD-EC011D43C15E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE495C9F-DD90-4710-8D27-4A2F27D2F19E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{DE495C9F-DD90-4710-8D27-4A2F27D2F19E}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo Físico" sheetId="11" r:id="rId1"/>
@@ -484,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -547,6 +547,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -565,12 +571,7 @@
     <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -915,20 +916,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="24"/>
+      <c r="B1" s="26"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -1014,14 +1015,14 @@
         <v>4</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -1049,10 +1050,10 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="1"/>
       <c r="D7" s="16">
         <v>1</v>
@@ -1267,10 +1268,10 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="26"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1288,13 +1289,13 @@
         <v>42</v>
       </c>
       <c r="C16" s="1"/>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
@@ -1392,14 +1393,14 @@
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -1440,7 +1441,7 @@
         <v>2</v>
       </c>
       <c r="G23" s="8">
-        <v>43881.625</v>
+        <v>46023.541666666664</v>
       </c>
       <c r="H23" s="7">
         <v>2</v>
@@ -1462,7 +1463,7 @@
         <v>2</v>
       </c>
       <c r="G24" s="8">
-        <v>43836.416666666664</v>
+        <v>46055.583333333336</v>
       </c>
       <c r="H24" s="7">
         <v>3</v>
@@ -1484,7 +1485,7 @@
         <v>2</v>
       </c>
       <c r="G25" s="8">
-        <v>43868.458333333336</v>
+        <v>46084.625</v>
       </c>
       <c r="H25" s="7">
         <v>2</v>
@@ -1506,7 +1507,7 @@
         <v>3</v>
       </c>
       <c r="G26" s="8">
-        <v>43137.416666666664</v>
+        <v>46116.666666666664</v>
       </c>
       <c r="H26" s="7">
         <v>2</v>
@@ -1528,7 +1529,7 @@
         <v>3</v>
       </c>
       <c r="G27" s="8">
-        <v>43503.458333333336</v>
+        <v>46147.708333333336</v>
       </c>
       <c r="H27" s="7">
         <v>3</v>
@@ -1550,7 +1551,7 @@
         <v>2</v>
       </c>
       <c r="G28" s="8">
-        <v>43898.625</v>
+        <v>46179.75</v>
       </c>
       <c r="H28" s="7">
         <v>1</v>
@@ -1572,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="G29" s="8">
-        <v>43899.458333333336</v>
+        <v>46210.791666666664</v>
       </c>
       <c r="H29" s="7">
         <v>1</v>
@@ -1596,14 +1597,14 @@
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
-      <c r="D31" s="29" t="s">
+      <c r="D31" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="29"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
       <c r="J31" s="1"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
@@ -1637,13 +1638,13 @@
         <v>3</v>
       </c>
       <c r="F33" s="9">
-        <v>1134567654</v>
+        <v>11911111111</v>
       </c>
       <c r="G33" s="9">
-        <v>435225435</v>
+        <v>111111111</v>
       </c>
       <c r="H33" s="9">
-        <v>94839859000</v>
+        <v>11111111111</v>
       </c>
       <c r="I33" s="9" t="s">
         <v>17</v>
@@ -1659,13 +1660,13 @@
         <v>4</v>
       </c>
       <c r="F34" s="9">
-        <v>11987656543</v>
+        <v>11922222222</v>
       </c>
       <c r="G34" s="9">
-        <v>326543457</v>
+        <v>222222222</v>
       </c>
       <c r="H34" s="9">
-        <v>73556944057</v>
+        <v>22222222222</v>
       </c>
       <c r="I34" s="9" t="s">
         <v>18</v>
@@ -1681,13 +1682,13 @@
         <v>5</v>
       </c>
       <c r="F35" s="9">
-        <v>11972084453</v>
+        <v>11933333333</v>
       </c>
       <c r="G35" s="9">
-        <v>546365253</v>
+        <v>333333333</v>
       </c>
       <c r="H35" s="9">
-        <v>16839338002</v>
+        <v>33333333333</v>
       </c>
       <c r="I35" s="9" t="s">
         <v>19</v>
@@ -1703,13 +1704,13 @@
         <v>6</v>
       </c>
       <c r="F36" s="9">
-        <v>1134566543</v>
+        <v>11944444444</v>
       </c>
       <c r="G36" s="9">
-        <v>543663625</v>
+        <v>444444444</v>
       </c>
       <c r="H36" s="9">
-        <v>14332654765</v>
+        <v>44444444444</v>
       </c>
       <c r="I36" s="9" t="s">
         <v>20</v>
@@ -1726,10 +1727,10 @@
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9">
-        <v>545662668</v>
+        <v>555555555</v>
       </c>
       <c r="H37" s="9">
-        <v>13771913039</v>
+        <v>55555555555</v>
       </c>
       <c r="I37" s="9" t="s">
         <v>21</v>
@@ -1801,15 +1802,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
@@ -1876,10 +1877,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="24"/>
+      <c r="B1" s="26"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -1931,10 +1932,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="28"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
@@ -1986,10 +1987,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="22"/>
+      <c r="B1" s="24"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
@@ -2061,14 +2062,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
@@ -2281,13 +2282,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
@@ -2363,14 +2364,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:8" x14ac:dyDescent="0.3">
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C2" s="20" t="s">
@@ -2400,13 +2401,13 @@
         <v>3</v>
       </c>
       <c r="E3" s="9">
-        <v>1134567654</v>
+        <v>11911111111</v>
       </c>
       <c r="F3" s="9">
-        <v>435225435</v>
+        <v>111111111</v>
       </c>
       <c r="G3" s="9">
-        <v>94839859000</v>
+        <v>11111111111</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>17</v>
@@ -2420,13 +2421,13 @@
         <v>4</v>
       </c>
       <c r="E4" s="9">
-        <v>11987656543</v>
+        <v>11922222222</v>
       </c>
       <c r="F4" s="9">
-        <v>326543457</v>
+        <v>222222222</v>
       </c>
       <c r="G4" s="9">
-        <v>73556944057</v>
+        <v>22222222222</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>18</v>
@@ -2440,13 +2441,13 @@
         <v>5</v>
       </c>
       <c r="E5" s="9">
-        <v>11972084453</v>
+        <v>11933333333</v>
       </c>
       <c r="F5" s="9">
-        <v>546365253</v>
+        <v>333333333</v>
       </c>
       <c r="G5" s="9">
-        <v>16839338002</v>
+        <v>33333333333</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>19</v>
@@ -2460,13 +2461,13 @@
         <v>6</v>
       </c>
       <c r="E6" s="9">
-        <v>1134566543</v>
+        <v>11944444444</v>
       </c>
       <c r="F6" s="9">
-        <v>543663625</v>
+        <v>444444444</v>
       </c>
       <c r="G6" s="9">
-        <v>14332654765</v>
+        <v>44444444444</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>20</v>
@@ -2481,10 +2482,10 @@
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9">
-        <v>545662668</v>
+        <v>555555555</v>
       </c>
       <c r="G7" s="9">
-        <v>13771913039</v>
+        <v>55555555555</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>21</v>
@@ -2500,7 +2501,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687E9CC1-5BE2-4E55-AEB6-B95901EDF055}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="10.109375" bestFit="1" customWidth="1"/>
@@ -2510,14 +2511,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
@@ -2550,7 +2551,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="8">
-        <v>43881.625</v>
+        <v>46023.541666666664</v>
       </c>
       <c r="E3" s="7">
         <v>2</v>
@@ -2568,7 +2569,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="8">
-        <v>43836.416666666664</v>
+        <v>46055.583333333336</v>
       </c>
       <c r="E4" s="7">
         <v>3</v>
@@ -2586,7 +2587,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="8">
-        <v>43868.458333333336</v>
+        <v>46084.625</v>
       </c>
       <c r="E5" s="7">
         <v>2</v>
@@ -2604,7 +2605,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="8">
-        <v>43137.416666666664</v>
+        <v>46116.666666666664</v>
       </c>
       <c r="E6" s="7">
         <v>2</v>
@@ -2622,7 +2623,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="8">
-        <v>43503.458333333336</v>
+        <v>46147.708333333336</v>
       </c>
       <c r="E7" s="7">
         <v>3</v>
@@ -2640,7 +2641,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="8">
-        <v>43898.625</v>
+        <v>46179.75</v>
       </c>
       <c r="E8" s="7">
         <v>1</v>
@@ -2658,17 +2659,21 @@
         <v>3</v>
       </c>
       <c r="D9" s="8">
-        <v>43899.458333333336</v>
+        <v>46210.791666666664</v>
       </c>
       <c r="E9" s="7">
         <v>1</v>
       </c>
       <c r="F9" s="7"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C11" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>